<commit_message>
docs(graph_app): add challenge-and-solution Q&A for TS migration
Frugal replace-not-port, Dart+TS coexistence without migrating graph_ui first, and 13 related decisions for a manager briefing.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/graph_app/graph_app-ts-migration-manager-briefing.xlsx
+++ b/graph_app/graph_app-ts-migration-manager-briefing.xlsx
@@ -8,31 +8,33 @@
   </bookViews>
   <sheets>
     <sheet name="00-Snapshot" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="01-How to use this sheet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="02-Ask of manager" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="03-Complexities" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="04-Challenges" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="05-Blockers and risks" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="06-Recommended POC" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="07-Open questions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="01-Challenge and solution" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="01-How to use this sheet" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="02-Ask of manager" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="03-Complexities" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="04-Challenges" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="05-Blockers and risks" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="06-Recommended POC" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="07-Open questions" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00-Snapshot'!$A$5:$D$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'00-Snapshot'!$1:$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01-How to use this sheet'!$A$19:$D$19</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'01-How to use this sheet'!$1:$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02-Ask of manager'!$A$5:$G$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'02-Ask of manager'!$1:$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03-Complexities'!$A$5:$H$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'03-Complexities'!$1:$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04-Challenges'!$A$5:$G$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'04-Challenges'!$1:$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05-Blockers and risks'!$A$5:$G$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'05-Blockers and risks'!$1:$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06-Recommended POC'!$A$10:$B$10</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'06-Recommended POC'!$1:$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07-Open questions'!$A$5:$E$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'07-Open questions'!$1:$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01-Challenge and solution'!$A$5:$E$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'01-How to use this sheet'!$A$19:$D$19</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'01-How to use this sheet'!$1:$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'02-Ask of manager'!$A$5:$G$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'02-Ask of manager'!$1:$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'03-Complexities'!$A$5:$H$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'03-Complexities'!$1:$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'04-Challenges'!$A$5:$G$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'04-Challenges'!$1:$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'05-Blockers and risks'!$A$5:$G$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'05-Blockers and risks'!$1:$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'06-Recommended POC'!$A$10:$B$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'06-Recommended POC'!$1:$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'07-Open questions'!$A$5:$E$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'07-Open questions'!$1:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -41,7 +43,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -118,6 +120,17 @@
       <color rgb="001E8449"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F6C8C"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -183,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -223,6 +236,25 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -820,7 +852,7 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Recommended ask in the meeting</t>
+          <t>Recommended ask in the meeting (see also tab 01-Challenge and solution)</t>
         </is>
       </c>
     </row>
@@ -859,6 +891,465 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Challenges and solutions (the list to share)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Each row is one decision in Q&amp;A form: the challenge, whether we migrate that layer, and the solution. Start with rows 1 and 2 in the meeting (Frugal, and Dart+TypeScript without moving graph_ui).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>graph_app (w_sox)  |  26 Aug 2026  |  Full prose: challenges-and-solutions.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Challenge (the question)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Do we migrate this layer?</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Solution</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>In first POC?</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="88" customHeight="1">
+      <c r="A6" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Frugal / NATS: how do we do this in TypeScript? Do we migrate Frugal, or move to something else?</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>No — do not port Frugal to TypeScript</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Org: Frugal is not supported in TS. ts-grc already replaced it with GraphQL (Apollo) + REST (RTK Query), and polling instead of NATS pub/sub. For SOX: keep Dart GraphModule / export streams until evergreen or graph-rpc exposes GraphQL/REST. Optional: Dart calls Frugal and passes JSON/props to TS. TS never imports frugal.</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>No NATS. POC-2 = one REST or GraphQL call only</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="88" customHeight="1">
+      <c r="A7" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Can Dart and TypeScript run together? Can we migrate graph_app without migrating graph_ui and other Dart packages?</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Yes, coexist. No, do not migrate graph_ui first</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>WDesk stays Dart and still loads w_sox. TypeScript cannot import Dart packages (graph_ui, audit, w_table, w_graph_client). TS screens must not call graph_ui. Leave graph_ui/audit/w_table as Dart islands. Migrate graph_app chrome that does not need graph_ui first (Support, simple dialogs, landing-widget chrome). A full TS graph_app is not possible until those islands have a TS/MFE home.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Yes — prove coexistence. No graph_ui in the widget</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="88" customHeight="1">
+      <c r="A8" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>WDesk is still Dart. How does TypeScript load? Can we put a TS package in WDesk pubspec?</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>No npm in Dart pubspec. Change the integration model</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Preferred: TypeScript MFE (ts-grc pattern) loaded from CDN at runtime. Fallback: Dart experience hosts a TS widget. Keep w_sox in WDesk pubspec until that screen is cut over. Do not build a standalone SOX website (loses login, nav, licensing).</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Yes — one load path only</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="88" customHeight="1">
+      <c r="A9" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>OverReact UI: is there a converter, or do we rewrite?</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Rewrite UI (no converter)</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Manual rewrite to React 18 + @workiva/unify (same as ts-grc). Do not use raw MUI as the long-term look. One small panel in the POC, not Testing or Reports.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>One Unify panel only</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="88" customHeight="1">
+      <c r="A10" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>State: Flux and Redux both exist. Can Dart and TS share one store?</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>No shared store</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Pass props/callbacks while hybrid. When a whole experience is TS, use Redux Toolkit local to that screen (ts-grc). Do not put the store on window. Port per experience, not globally.</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Presentational TS only (props)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="88" customHeight="1">
+      <c r="A11" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>w_table / smart table: must we migrate the grid before SOX TypeScript?</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>No — keep Dart island</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Highest UI cost. Plugins do not map 1:1. First TS screens must not include the grid. Revisit when platform has a TS grid.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Out of scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="88" customHeight="1">
+      <c r="A12" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Audit is compiled into SOX. Must we migrate Audit (and other product packages) first?</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>No — keep Audit as a Dart island</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>SOX cannot pub-get a TypeScript Audit package. Same for comments, attachments, viewer, drawing, spreadsheet. Analyze audit as its own repo. Future: Audit MFE. POC must not include Audit forms.</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Out of scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="88" customHeight="1">
+      <c r="A13" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Login, session, and licensing: does TypeScript own auth?</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>No new login. Reuse shell. Relicense carefully</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>WDesk owns the cookie. Use shell session (ts-grc: session MFE service). Experience canUserAccessV2 stays Dart until that screen is an MFE. Any customer-facing TS UI must match Dart ability + workspace rules (SOX vs ERM vs ESG). Compliance gate, not polish.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Reuse session. Do not change access rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="88" customHeight="1">
+      <c r="A14" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>LaunchDarkly: new flags for TypeScript?</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>Replace SDK only — same flag keys</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Use @workiva/grc-launch-darkly. Keep existing keys so Dart and TS dual-run. Do not invent parallel flags.</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Yes — one existing flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="88" customHeight="1">
+      <c r="A15" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Models (built_value, GRC YAML): convert all models first?</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>No bulk dump — port with each screen</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>No .sg.dart→TS converter. Later generate TS from the same grc_model.yaml as Dart. POC does not migrate the model layer.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Out of scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="88" customHeight="1">
+      <c r="A16" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Tests: port unit and Skynet functional tests first?</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>Unit with each widget. Functional tests not first</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Vitest + Testing Library in the same PR as the TS widget. Keep Dart unit tests until that Dart screen is deleted. Keep Puppeteer/Skynet green. Playwright later after dual-run. Do not spend the POC rewriting functional tests.</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>One unit test. Do not port Skynet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="88" customHeight="1">
+      <c r="A17" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Deploy: replace dart2js CDN / FEWS / pub package?</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>Add a TS artifact later — do not replace Dart deploy for the POC</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>POC uses current Dart CDN/FEWS. A real TS MFE gets its own pipeline (ts-grc). Dual deploy until that Dart experience is removed. Rollback = Dart.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Use existing Dart deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="88" customHeight="1">
+      <c r="A18" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>i18n, analytics, logging: new event names and hardcoded strings?</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>Reuse Workiva TS packages; keep Next Gen analytics names</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>w_intl_ts + react-intl (no hardcoded UI text). Analytics: names from ANALYTICS_MIGRATION_MAPPING.md. Logging: grc-logger; TS errors must reach App Intelligence.</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Optional: one log/error boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="88" customHeight="1">
+      <c r="A19" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Comments, attachments, viewer, drawing, spreadsheet: replace with generic npm libraries?</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>No — platform Dart/MFE islands</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Dart experience keeps loading those CSS/JS assets. Do not replace w_viewer with a generic PDF viewer or the spreadsheet with a generic grid.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Out of scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="88" customHeight="1">
+      <c r="A20" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Landing widgets and embeddable spreadsheets: can we remove w_sox from WDesk after one TS screen?</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="inlineStr">
+        <is>
+          <t>No — Dart keeps registering them until WDesk has an MFE contribution point</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Those configs still live on w_sox. Confirm widget/embeddable MFE support before promising to drop the Dart package.</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Out of scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>Meeting takeaway: (1) Do not port Frugal — replace with GraphQL/REST and keep Dart for NATS until coverage exists. (2) Yes, Dart+TS together — migrate graph_app chrome without moving graph_ui/audit/w_table. POC = one Unify widget + later one REST/GraphQL call.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:E20"/>
+  <mergeCells count="4">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="3" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D22"/>
@@ -1179,7 +1670,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1547,7 +2038,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2371,7 +2862,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2999,546 +3490,6 @@
       <c r="G20" s="6" t="inlineStr">
         <is>
           <t>Confirm where they register before promising bundle-size wins</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A5:G5"/>
-  <mergeCells count="3">
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;Lgraph_app Dart → TypeScript  |  Internal briefing</oddHeader>
-    <oddFooter>&amp;LNot a commitment to rewrite SOX. Next: living analysis in research-and-learnings.&amp;RPage &amp;P of &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Blockers and risks</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Blocker = POC-2 or a full cutover cannot succeed until this has a path. Risk = can proceed but needs a control.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Repo analyzed: graph_app (published as w_sox)  |  Date: 25 Aug 2026  |  Audience: engineering manager  |  Status: pre-POC briefing — not a rewrite proposal</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Why it hurts</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Needed before</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Owner to assign</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Mitigation</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>WDesk Dart pubspec ↔ w_sox</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>A TypeScript package cannot replace w_sox without an MFE (or Dart facade).</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Any production TS SOX app</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>WDesk</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Keep Dart w_sox; add MFE or hybrid island.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>No TypeScript Frugal; SOX APIs still NATS</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>Graph, GRC services, export status still NATS. ts-grc GraphQL may not cover them.</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>POC-2 and any data-heavy screen</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>evergreen / graph API</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>Inventory GraphQL/REST; poll or keep Dart streams.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>B3</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>package:audit compiled in</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>SOX cannot be fully TS while Audit is a Dart library.</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Declaring SOX 'done' in TS</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Audit</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Dart island or Audit MFE later.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>B4</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>package:graph_ui compiled in</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Same as Audit for shared graph UI.</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Declaring SOX 'done' in TS</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>graph_ui</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Dart island; analyze graph_ui next.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>B5</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Licensing + workspace access rules</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Compliance incident if TS gates differ.</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Any customer-facing TS screen</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>GRC + licensing</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Golden tests Dart vs TS; no rule changes in POC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>High risk</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>w_table / smart table</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Highest UI cost; last to move.</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>Reports / test-step TS</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>w_table</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>Keep grid in Dart.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>High risk</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Two state systems + no shared Dart/TS store</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Hybrid screens disagree on data.</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Any hybrid feature</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>graph_app</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Props/callbacks only in POC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>High risk</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Dual deploy artifacts</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Harder rollback and version skew.</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Second TS artifact</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>DevOps</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>POC uses current Dart CDN/FEWS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>R4</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>High risk</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Skynet functional tests</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>False confidence if we skip; wasted time if we port first.</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Experience cutover</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>DevOps</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Keep Dart tests green.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>R5</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Analytics dual-send still in progress</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Metrics drop or duplicate.</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Any TS event</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Analytics</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>Next Gen names only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>R6</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Git-pinned audit / wdesk_sdk</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>POC can break on unrelated SHA bumps.</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>Release train</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>Platform</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Pin and communicate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>R7</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>User content XSS/CSP (forms, TQ, markup)</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Security regression.</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Any TS form</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>graph_app + Infosec</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>React escaping; no innerHTML; shell CSP.</t>
         </is>
       </c>
     </row>
@@ -3568,6 +3519,546 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Blockers and risks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Blocker = POC-2 or a full cutover cannot succeed until this has a path. Risk = can proceed but needs a control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Repo analyzed: graph_app (published as w_sox)  |  Date: 25 Aug 2026  |  Audience: engineering manager  |  Status: pre-POC briefing — not a rewrite proposal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Why it hurts</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Needed before</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Owner to assign</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Mitigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>WDesk Dart pubspec ↔ w_sox</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>A TypeScript package cannot replace w_sox without an MFE (or Dart facade).</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Any production TS SOX app</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>WDesk</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Keep Dart w_sox; add MFE or hybrid island.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>No TypeScript Frugal; SOX APIs still NATS</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Graph, GRC services, export status still NATS. ts-grc GraphQL may not cover them.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>POC-2 and any data-heavy screen</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>evergreen / graph API</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Inventory GraphQL/REST; poll or keep Dart streams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>package:audit compiled in</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>SOX cannot be fully TS while Audit is a Dart library.</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Declaring SOX 'done' in TS</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Audit</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Dart island or Audit MFE later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>package:graph_ui compiled in</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Same as Audit for shared graph UI.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Declaring SOX 'done' in TS</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>graph_ui</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Dart island; analyze graph_ui next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Licensing + workspace access rules</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Compliance incident if TS gates differ.</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Any customer-facing TS screen</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>GRC + licensing</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Golden tests Dart vs TS; no rule changes in POC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>High risk</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>w_table / smart table</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Highest UI cost; last to move.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Reports / test-step TS</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>w_table</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Keep grid in Dart.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>High risk</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Two state systems + no shared Dart/TS store</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Hybrid screens disagree on data.</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Any hybrid feature</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>graph_app</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Props/callbacks only in POC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>High risk</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Dual deploy artifacts</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Harder rollback and version skew.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Second TS artifact</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>POC uses current Dart CDN/FEWS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>High risk</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Skynet functional tests</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>False confidence if we skip; wasted time if we port first.</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Experience cutover</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Keep Dart tests green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Analytics dual-send still in progress</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Metrics drop or duplicate.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Any TS event</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Next Gen names only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Git-pinned audit / wdesk_sdk</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>POC can break on unrelated SHA bumps.</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Release train</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Pin and communicate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>User content XSS/CSP (forms, TQ, markup)</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Security regression.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Any TS form</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>graph_app + Infosec</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>React escaping; no innerHTML; shell CSP.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:G5"/>
+  <mergeCells count="3">
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;Lgraph_app Dart → TypeScript  |  Internal briefing</oddHeader>
+    <oddFooter>&amp;LNot a commitment to rewrite SOX. Next: living analysis in research-and-learnings.&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3816,7 +4307,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs(graph_app): explain hybrid Dart+TS deploy is not microservices
POC ships TypeScript as JS on the existing CDN; a later MFE is a second frontend artifact, not a new backend service per screen.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/graph_app/graph_app-ts-migration-manager-briefing.xlsx
+++ b/graph_app/graph_app-ts-migration-manager-briefing.xlsx
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00-Snapshot'!$A$5:$D$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'00-Snapshot'!$1:$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01-Challenge and solution'!$A$5:$E$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01-Challenge and solution'!$A$5:$E$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'01-How to use this sheet'!$A$19:$D$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'01-How to use this sheet'!$1:$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'02-Ask of manager'!$A$5:$G$5</definedName>
@@ -196,7 +196,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -255,6 +255,9 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -893,7 +896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1326,19 +1329,47 @@
         </is>
       </c>
     </row>
+    <row r="21" ht="96" customHeight="1">
+      <c r="A21" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Dart + TypeScript in the same product: how do we deploy? Do we need everything as a microservice?</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>No — not microservices. Frontend packaging only</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>MFE ≠ microservice. Backends stay as they are. POC Model A: Vite builds JS, include it in the existing w_sox/CDN tarball (same way graph_app already loads graph_app_js). Later Model B: a TS MFE is a second FEWS/CDN frontend artifact next to Dart w_sox; WDesk loads both. Do not create a K8s service per screen or a new Frugal service for TypeScript.</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Model A: JS on existing Dart CDN</t>
+        </is>
+      </c>
+    </row>
     <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="22" t="inlineStr">
-        <is>
-          <t>Meeting takeaway: (1) Do not port Frugal — replace with GraphQL/REST and keep Dart for NATS until coverage exists. (2) Yes, Dart+TS together — migrate graph_app chrome without moving graph_ui/audit/w_table. POC = one Unify widget + later one REST/GraphQL call.</t>
+      <c r="A22" s="22" t="n"/>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>Meeting takeaway: (1) Do not port Frugal — replace with GraphQL/REST and keep Dart for NATS until coverage exists. (2) Yes, Dart+TS together — migrate graph_app chrome without moving graph_ui/audit/w_table. POC = one Unify widget + later one REST/GraphQL call. Deploy is not microservices: POC ships TS as JS on the existing CDN, or later as one TS MFE artifact beside w_sox.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:E20"/>
+  <autoFilter ref="A5:E21"/>
   <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A22:E22"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A23:E23"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>